<commit_message>
_calibration for protein solution
</commit_message>
<xml_diff>
--- a/zeus-pipetter/calibration_for_pipetting/pipetting_calibration_substances.xlsx
+++ b/zeus-pipetter/calibration_for_pipetting/pipetting_calibration_substances.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chemiluminescence\OneDrive\roborea\zeus-pipetter\calibration_for_pipetting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80B4E16-3BE5-4A0A-843C-AA10546237D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F0B17C-152C-42A3-9418-817B4B2977BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6AD12529-BA13-4E6D-84B7-065B2794C4B4}"/>
   </bookViews>
@@ -34,18 +34,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>PBS</t>
+    <t>reaction_id</t>
+  </si>
+  <si>
+    <t>FBS</t>
   </si>
   <si>
     <t>DMEM</t>
   </si>
   <si>
-    <t>BSA_32uM</t>
+    <t>BSA32</t>
   </si>
   <si>
-    <t>reaction_id</t>
+    <t>LZ32</t>
+  </si>
+  <si>
+    <t>NP_MUA</t>
   </si>
 </sst>
 </file>
@@ -420,34 +426,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D452BF46-4201-4845-9E78-8B75FAF11789}">
-  <dimension ref="A1:O88"/>
+  <dimension ref="A1:M94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" customWidth="1"/>
-    <col min="6" max="7" width="10.28515625" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" customWidth="1"/>
-    <col min="11" max="11" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="5" width="10.28515625" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -455,15 +464,13 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-    </row>
-    <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -476,15 +483,13 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-    </row>
-    <row r="3" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>200</v>
+        <v>20</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -497,15 +502,13 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-    </row>
-    <row r="4" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="1">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -518,17 +521,15 @@
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-    </row>
-    <row r="5" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1">
-        <v>10</v>
-      </c>
+      <c r="B5" s="1">
+        <v>50</v>
+      </c>
+      <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -539,17 +540,15 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-    </row>
-    <row r="6" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1">
-        <v>20</v>
-      </c>
+      <c r="B6" s="1">
+        <v>75</v>
+      </c>
+      <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -560,17 +559,15 @@
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-    </row>
-    <row r="7" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1">
-        <v>30</v>
-      </c>
+      <c r="B7" s="1">
+        <v>100</v>
+      </c>
+      <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -581,18 +578,16 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-    </row>
-    <row r="8" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="1"/>
+      <c r="B8" s="1">
+        <v>200</v>
+      </c>
       <c r="C8" s="1"/>
-      <c r="D8" s="1">
-        <v>10</v>
-      </c>
+      <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -602,18 +597,16 @@
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-    </row>
-    <row r="9" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="1"/>
+      <c r="B9" s="1">
+        <v>300</v>
+      </c>
       <c r="C9" s="1"/>
-      <c r="D9" s="1">
-        <v>20</v>
-      </c>
+      <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
@@ -623,18 +616,15 @@
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-    </row>
-    <row r="10" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1">
-        <v>30</v>
-      </c>
+      <c r="C10" s="1">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
@@ -644,13 +634,14 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-    </row>
-    <row r="11" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
+    </row>
+    <row r="11" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>9</v>
+      </c>
+      <c r="C11" s="1">
+        <v>20</v>
+      </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -661,13 +652,14 @@
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-    </row>
-    <row r="12" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+    </row>
+    <row r="12" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>10</v>
+      </c>
+      <c r="C12" s="1">
+        <v>30</v>
+      </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -678,13 +670,14 @@
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-    </row>
-    <row r="13" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+    </row>
+    <row r="13" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>11</v>
+      </c>
+      <c r="C13" s="1">
+        <v>50</v>
+      </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -695,13 +688,14 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-    </row>
-    <row r="14" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+    </row>
+    <row r="14" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1">
+        <v>75</v>
+      </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
@@ -712,13 +706,14 @@
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-    </row>
-    <row r="15" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+    </row>
+    <row r="15" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>13</v>
+      </c>
+      <c r="C15" s="1">
+        <v>100</v>
+      </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -729,13 +724,14 @@
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-    </row>
-    <row r="16" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+    </row>
+    <row r="16" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>14</v>
+      </c>
+      <c r="C16" s="1">
+        <v>200</v>
+      </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -746,13 +742,14 @@
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-    </row>
-    <row r="17" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+    </row>
+    <row r="17" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>15</v>
+      </c>
+      <c r="C17" s="1">
+        <v>300</v>
+      </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -763,14 +760,14 @@
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-    </row>
-    <row r="18" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -780,14 +777,14 @@
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-    </row>
-    <row r="19" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
+      <c r="D19" s="1">
+        <v>2</v>
+      </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -797,14 +794,14 @@
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-    </row>
-    <row r="20" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
+      <c r="D20" s="1">
+        <v>5</v>
+      </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -814,14 +811,14 @@
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-    </row>
-    <row r="21" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
+      <c r="D21" s="1">
+        <v>7.5</v>
+      </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
@@ -831,14 +828,14 @@
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-    </row>
-    <row r="22" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
+      <c r="D22" s="1">
+        <v>10</v>
+      </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
@@ -848,14 +845,14 @@
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-    </row>
-    <row r="23" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
+      <c r="D23" s="1">
+        <v>20</v>
+      </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
@@ -865,14 +862,14 @@
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-    </row>
-    <row r="24" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
+      <c r="D24" s="1">
+        <v>30</v>
+      </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
@@ -882,14 +879,14 @@
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-    </row>
-    <row r="25" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
+      <c r="D25" s="1">
+        <v>50</v>
+      </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
@@ -899,15 +896,15 @@
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-    </row>
-    <row r="26" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
+      <c r="E26" s="1">
+        <v>1</v>
+      </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
@@ -916,15 +913,15 @@
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-    </row>
-    <row r="27" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
+      <c r="E27" s="1">
+        <v>2</v>
+      </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
@@ -933,15 +930,15 @@
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1"/>
-    </row>
-    <row r="28" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
+      <c r="E28" s="1">
+        <v>5</v>
+      </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
@@ -950,15 +947,15 @@
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
-      <c r="O28" s="1"/>
-    </row>
-    <row r="29" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
+      <c r="E29" s="1">
+        <v>7.5</v>
+      </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
@@ -967,15 +964,15 @@
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-    </row>
-    <row r="30" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
+      <c r="E30" s="1">
+        <v>10</v>
+      </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
@@ -984,15 +981,15 @@
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-    </row>
-    <row r="31" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
+      <c r="E31" s="1">
+        <v>20</v>
+      </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
@@ -1001,15 +998,15 @@
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-    </row>
-    <row r="32" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
+      <c r="E32" s="1">
+        <v>30</v>
+      </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
@@ -1018,15 +1015,15 @@
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
-      <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
-    </row>
-    <row r="33" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
+      <c r="E33" s="1">
+        <v>50</v>
+      </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
@@ -1035,16 +1032,16 @@
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-    </row>
-    <row r="34" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
+      <c r="F34" s="1">
+        <v>1</v>
+      </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
@@ -1052,16 +1049,16 @@
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-    </row>
-    <row r="35" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
+      <c r="F35" s="1">
+        <v>2</v>
+      </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
@@ -1069,16 +1066,16 @@
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
-      <c r="N35" s="1"/>
-      <c r="O35" s="1"/>
-    </row>
-    <row r="36" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
+      <c r="F36" s="1">
+        <v>5</v>
+      </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
@@ -1086,16 +1083,16 @@
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-    </row>
-    <row r="37" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
+      <c r="F37" s="1">
+        <v>7.5</v>
+      </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
@@ -1103,16 +1100,16 @@
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
-    </row>
-    <row r="38" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
+      <c r="F38" s="1">
+        <v>10</v>
+      </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -1120,16 +1117,16 @@
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
-    </row>
-    <row r="39" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
+      <c r="F39" s="1">
+        <v>20</v>
+      </c>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
@@ -1137,16 +1134,16 @@
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
-      <c r="N39" s="1"/>
-      <c r="O39" s="1"/>
-    </row>
-    <row r="40" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
+      <c r="F40" s="1">
+        <v>30</v>
+      </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
@@ -1154,16 +1151,16 @@
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
-      <c r="N40" s="1"/>
-      <c r="O40" s="1"/>
-    </row>
-    <row r="41" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
+      <c r="F41" s="1">
+        <v>50</v>
+      </c>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
@@ -1171,10 +1168,8 @@
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
-    </row>
-    <row r="42" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -1188,10 +1183,8 @@
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1"/>
-    </row>
-    <row r="43" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1205,10 +1198,8 @@
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
-      <c r="N43" s="1"/>
-      <c r="O43" s="1"/>
-    </row>
-    <row r="44" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1222,10 +1213,8 @@
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
-      <c r="N44" s="1"/>
-      <c r="O44" s="1"/>
-    </row>
-    <row r="45" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -1239,10 +1228,8 @@
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
-      <c r="N45" s="1"/>
-      <c r="O45" s="1"/>
-    </row>
-    <row r="46" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1256,10 +1243,8 @@
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
-      <c r="N46" s="1"/>
-      <c r="O46" s="1"/>
-    </row>
-    <row r="47" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1273,10 +1258,8 @@
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
-      <c r="N47" s="1"/>
-      <c r="O47" s="1"/>
-    </row>
-    <row r="48" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -1290,10 +1273,8 @@
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
-      <c r="N48" s="1"/>
-      <c r="O48" s="1"/>
-    </row>
-    <row r="49" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -1307,10 +1288,8 @@
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
-      <c r="N49" s="1"/>
-      <c r="O49" s="1"/>
-    </row>
-    <row r="50" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -1324,10 +1303,8 @@
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
-      <c r="N50" s="1"/>
-      <c r="O50" s="1"/>
-    </row>
-    <row r="51" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="51" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -1341,10 +1318,8 @@
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
-      <c r="N51" s="1"/>
-      <c r="O51" s="1"/>
-    </row>
-    <row r="52" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1358,10 +1333,8 @@
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
-      <c r="N52" s="1"/>
-      <c r="O52" s="1"/>
-    </row>
-    <row r="53" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="53" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1375,10 +1348,8 @@
       <c r="K53" s="1"/>
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
-      <c r="N53" s="1"/>
-      <c r="O53" s="1"/>
-    </row>
-    <row r="54" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -1392,10 +1363,8 @@
       <c r="K54" s="1"/>
       <c r="L54" s="1"/>
       <c r="M54" s="1"/>
-      <c r="N54" s="1"/>
-      <c r="O54" s="1"/>
-    </row>
-    <row r="55" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="55" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -1409,10 +1378,8 @@
       <c r="K55" s="1"/>
       <c r="L55" s="1"/>
       <c r="M55" s="1"/>
-      <c r="N55" s="1"/>
-      <c r="O55" s="1"/>
-    </row>
-    <row r="56" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -1426,10 +1393,8 @@
       <c r="K56" s="1"/>
       <c r="L56" s="1"/>
       <c r="M56" s="1"/>
-      <c r="N56" s="1"/>
-      <c r="O56" s="1"/>
-    </row>
-    <row r="57" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="57" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -1443,10 +1408,8 @@
       <c r="K57" s="1"/>
       <c r="L57" s="1"/>
       <c r="M57" s="1"/>
-      <c r="N57" s="1"/>
-      <c r="O57" s="1"/>
-    </row>
-    <row r="58" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="58" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -1460,10 +1423,8 @@
       <c r="K58" s="1"/>
       <c r="L58" s="1"/>
       <c r="M58" s="1"/>
-      <c r="N58" s="1"/>
-      <c r="O58" s="1"/>
-    </row>
-    <row r="59" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="59" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -1477,10 +1438,8 @@
       <c r="K59" s="1"/>
       <c r="L59" s="1"/>
       <c r="M59" s="1"/>
-      <c r="N59" s="1"/>
-      <c r="O59" s="1"/>
-    </row>
-    <row r="60" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="60" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -1494,10 +1453,8 @@
       <c r="K60" s="1"/>
       <c r="L60" s="1"/>
       <c r="M60" s="1"/>
-      <c r="N60" s="1"/>
-      <c r="O60" s="1"/>
-    </row>
-    <row r="61" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="61" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -1511,10 +1468,8 @@
       <c r="K61" s="1"/>
       <c r="L61" s="1"/>
       <c r="M61" s="1"/>
-      <c r="N61" s="1"/>
-      <c r="O61" s="1"/>
-    </row>
-    <row r="62" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="62" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -1528,10 +1483,8 @@
       <c r="K62" s="1"/>
       <c r="L62" s="1"/>
       <c r="M62" s="1"/>
-      <c r="N62" s="1"/>
-      <c r="O62" s="1"/>
-    </row>
-    <row r="63" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="63" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -1545,10 +1498,8 @@
       <c r="K63" s="1"/>
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
-      <c r="N63" s="1"/>
-      <c r="O63" s="1"/>
-    </row>
-    <row r="64" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="64" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -1562,10 +1513,8 @@
       <c r="K64" s="1"/>
       <c r="L64" s="1"/>
       <c r="M64" s="1"/>
-      <c r="N64" s="1"/>
-      <c r="O64" s="1"/>
-    </row>
-    <row r="65" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="65" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -1579,10 +1528,8 @@
       <c r="K65" s="1"/>
       <c r="L65" s="1"/>
       <c r="M65" s="1"/>
-      <c r="N65" s="1"/>
-      <c r="O65" s="1"/>
-    </row>
-    <row r="66" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="66" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -1596,10 +1543,8 @@
       <c r="K66" s="1"/>
       <c r="L66" s="1"/>
       <c r="M66" s="1"/>
-      <c r="N66" s="1"/>
-      <c r="O66" s="1"/>
-    </row>
-    <row r="67" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="67" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -1613,10 +1558,8 @@
       <c r="K67" s="1"/>
       <c r="L67" s="1"/>
       <c r="M67" s="1"/>
-      <c r="N67" s="1"/>
-      <c r="O67" s="1"/>
-    </row>
-    <row r="68" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="68" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -1630,10 +1573,8 @@
       <c r="K68" s="1"/>
       <c r="L68" s="1"/>
       <c r="M68" s="1"/>
-      <c r="N68" s="1"/>
-      <c r="O68" s="1"/>
-    </row>
-    <row r="69" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="69" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -1647,10 +1588,8 @@
       <c r="K69" s="1"/>
       <c r="L69" s="1"/>
       <c r="M69" s="1"/>
-      <c r="N69" s="1"/>
-      <c r="O69" s="1"/>
-    </row>
-    <row r="70" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="70" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -1664,10 +1603,8 @@
       <c r="K70" s="1"/>
       <c r="L70" s="1"/>
       <c r="M70" s="1"/>
-      <c r="N70" s="1"/>
-      <c r="O70" s="1"/>
-    </row>
-    <row r="71" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="71" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -1681,10 +1618,8 @@
       <c r="K71" s="1"/>
       <c r="L71" s="1"/>
       <c r="M71" s="1"/>
-      <c r="N71" s="1"/>
-      <c r="O71" s="1"/>
-    </row>
-    <row r="72" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="72" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -1698,10 +1633,8 @@
       <c r="K72" s="1"/>
       <c r="L72" s="1"/>
       <c r="M72" s="1"/>
-      <c r="N72" s="1"/>
-      <c r="O72" s="1"/>
-    </row>
-    <row r="73" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="73" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -1715,10 +1648,8 @@
       <c r="K73" s="1"/>
       <c r="L73" s="1"/>
       <c r="M73" s="1"/>
-      <c r="N73" s="1"/>
-      <c r="O73" s="1"/>
-    </row>
-    <row r="74" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="74" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -1732,10 +1663,8 @@
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
       <c r="M74" s="1"/>
-      <c r="N74" s="1"/>
-      <c r="O74" s="1"/>
-    </row>
-    <row r="75" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="75" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -1749,10 +1678,8 @@
       <c r="K75" s="1"/>
       <c r="L75" s="1"/>
       <c r="M75" s="1"/>
-      <c r="N75" s="1"/>
-      <c r="O75" s="1"/>
-    </row>
-    <row r="76" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="76" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -1766,10 +1693,8 @@
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
       <c r="M76" s="1"/>
-      <c r="N76" s="1"/>
-      <c r="O76" s="1"/>
-    </row>
-    <row r="77" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="77" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -1783,10 +1708,8 @@
       <c r="K77" s="1"/>
       <c r="L77" s="1"/>
       <c r="M77" s="1"/>
-      <c r="N77" s="1"/>
-      <c r="O77" s="1"/>
-    </row>
-    <row r="78" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="78" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -1800,10 +1723,8 @@
       <c r="K78" s="1"/>
       <c r="L78" s="1"/>
       <c r="M78" s="1"/>
-      <c r="N78" s="1"/>
-      <c r="O78" s="1"/>
-    </row>
-    <row r="79" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="79" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -1817,10 +1738,8 @@
       <c r="K79" s="1"/>
       <c r="L79" s="1"/>
       <c r="M79" s="1"/>
-      <c r="N79" s="1"/>
-      <c r="O79" s="1"/>
-    </row>
-    <row r="80" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="80" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -1834,10 +1753,8 @@
       <c r="K80" s="1"/>
       <c r="L80" s="1"/>
       <c r="M80" s="1"/>
-      <c r="N80" s="1"/>
-      <c r="O80" s="1"/>
-    </row>
-    <row r="81" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="81" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -1851,10 +1768,8 @@
       <c r="K81" s="1"/>
       <c r="L81" s="1"/>
       <c r="M81" s="1"/>
-      <c r="N81" s="1"/>
-      <c r="O81" s="1"/>
-    </row>
-    <row r="82" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="82" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -1868,10 +1783,8 @@
       <c r="K82" s="1"/>
       <c r="L82" s="1"/>
       <c r="M82" s="1"/>
-      <c r="N82" s="1"/>
-      <c r="O82" s="1"/>
-    </row>
-    <row r="83" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="83" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -1885,10 +1798,8 @@
       <c r="K83" s="1"/>
       <c r="L83" s="1"/>
       <c r="M83" s="1"/>
-      <c r="N83" s="1"/>
-      <c r="O83" s="1"/>
-    </row>
-    <row r="84" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="84" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -1902,10 +1813,8 @@
       <c r="K84" s="1"/>
       <c r="L84" s="1"/>
       <c r="M84" s="1"/>
-      <c r="N84" s="1"/>
-      <c r="O84" s="1"/>
-    </row>
-    <row r="85" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="85" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -1919,10 +1828,8 @@
       <c r="K85" s="1"/>
       <c r="L85" s="1"/>
       <c r="M85" s="1"/>
-      <c r="N85" s="1"/>
-      <c r="O85" s="1"/>
-    </row>
-    <row r="86" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="86" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -1936,10 +1843,8 @@
       <c r="K86" s="1"/>
       <c r="L86" s="1"/>
       <c r="M86" s="1"/>
-      <c r="N86" s="1"/>
-      <c r="O86" s="1"/>
-    </row>
-    <row r="87" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="87" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -1953,10 +1858,8 @@
       <c r="K87" s="1"/>
       <c r="L87" s="1"/>
       <c r="M87" s="1"/>
-      <c r="N87" s="1"/>
-      <c r="O87" s="1"/>
-    </row>
-    <row r="88" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="88" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -1970,8 +1873,96 @@
       <c r="K88" s="1"/>
       <c r="L88" s="1"/>
       <c r="M88" s="1"/>
-      <c r="N88" s="1"/>
-      <c r="O88" s="1"/>
+    </row>
+    <row r="89" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A89" s="1"/>
+      <c r="B89" s="1"/>
+      <c r="C89" s="1"/>
+      <c r="D89" s="1"/>
+      <c r="E89" s="1"/>
+      <c r="F89" s="1"/>
+      <c r="G89" s="1"/>
+      <c r="H89" s="1"/>
+      <c r="I89" s="1"/>
+      <c r="J89" s="1"/>
+      <c r="K89" s="1"/>
+      <c r="L89" s="1"/>
+      <c r="M89" s="1"/>
+    </row>
+    <row r="90" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A90" s="1"/>
+      <c r="B90" s="1"/>
+      <c r="C90" s="1"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+      <c r="F90" s="1"/>
+      <c r="G90" s="1"/>
+      <c r="H90" s="1"/>
+      <c r="I90" s="1"/>
+      <c r="J90" s="1"/>
+      <c r="K90" s="1"/>
+      <c r="L90" s="1"/>
+      <c r="M90" s="1"/>
+    </row>
+    <row r="91" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A91" s="1"/>
+      <c r="B91" s="1"/>
+      <c r="C91" s="1"/>
+      <c r="D91" s="1"/>
+      <c r="E91" s="1"/>
+      <c r="F91" s="1"/>
+      <c r="G91" s="1"/>
+      <c r="H91" s="1"/>
+      <c r="I91" s="1"/>
+      <c r="J91" s="1"/>
+      <c r="K91" s="1"/>
+      <c r="L91" s="1"/>
+      <c r="M91" s="1"/>
+    </row>
+    <row r="92" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A92" s="1"/>
+      <c r="B92" s="1"/>
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
+      <c r="F92" s="1"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="1"/>
+      <c r="I92" s="1"/>
+      <c r="J92" s="1"/>
+      <c r="K92" s="1"/>
+      <c r="L92" s="1"/>
+      <c r="M92" s="1"/>
+    </row>
+    <row r="93" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A93" s="1"/>
+      <c r="B93" s="1"/>
+      <c r="C93" s="1"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="1"/>
+      <c r="F93" s="1"/>
+      <c r="G93" s="1"/>
+      <c r="H93" s="1"/>
+      <c r="I93" s="1"/>
+      <c r="J93" s="1"/>
+      <c r="K93" s="1"/>
+      <c r="L93" s="1"/>
+      <c r="M93" s="1"/>
+    </row>
+    <row r="94" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A94" s="1"/>
+      <c r="B94" s="1"/>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+      <c r="F94" s="1"/>
+      <c r="G94" s="1"/>
+      <c r="H94" s="1"/>
+      <c r="I94" s="1"/>
+      <c r="J94" s="1"/>
+      <c r="K94" s="1"/>
+      <c r="L94" s="1"/>
+      <c r="M94" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>